<commit_message>
Ajusta proposta para R$ 541.360,00
Reduz gestão de 12% para 10%, revisa horas-base considerando recursos
nativos de Django/Wagtail (2.978 h -> 2.695 h) e ajusta a operação
(hospedagem R$ 1.300, backup R$ 640, suporte 15 h/mês).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W9k6rtJ9YG3B4ZzgCkiDqC
</commit_message>
<xml_diff>
--- a/docs/entregaveis/Observatorio_FBA_Precificacao_NatGED.xlsx
+++ b/docs/entregaveis/Observatorio_FBA_Precificacao_NatGED.xlsx
@@ -1091,7 +1091,7 @@
       </c>
       <c r="B5" s="5" t="n">
         <f aca="false">Componentes!$F$22</f>
-        <v>482480</v>
+        <v>437200</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1100,7 +1100,7 @@
       </c>
       <c r="B6" s="5" t="n">
         <f aca="false">Componentes!$F$28</f>
-        <v>132000</v>
+        <v>104160</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1109,7 +1109,7 @@
       </c>
       <c r="B7" s="7" t="n">
         <f aca="false">B5+B6</f>
-        <v>614480</v>
+        <v>541360</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1118,7 +1118,7 @@
       </c>
       <c r="B9" s="8" t="n">
         <f aca="false">Componentes!$D$22</f>
-        <v>2978</v>
+        <v>2695</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1127,7 +1127,7 @@
       </c>
       <c r="B10" s="5" t="n">
         <f aca="false">Componentes!$E$28</f>
-        <v>5500</v>
+        <v>4340</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1145,7 +1145,7 @@
       </c>
       <c r="B12" s="9" t="n">
         <f aca="false">B10*18</f>
-        <v>99000</v>
+        <v>78120</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1154,7 +1154,7 @@
       </c>
       <c r="B13" s="9" t="n">
         <f aca="false">B5+B12</f>
-        <v>581480</v>
+        <v>515320</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1230,7 +1230,7 @@
         <v>22</v>
       </c>
       <c r="B6" s="11" t="n">
-        <v>0.12</v>
+        <v>0.1</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>23</v>
@@ -1272,7 +1272,7 @@
         <v>31</v>
       </c>
       <c r="B9" s="12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>32</v>
@@ -1300,7 +1300,7 @@
         <v>37</v>
       </c>
       <c r="B11" s="12" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>32</v>
@@ -1380,7 +1380,7 @@
         <v>47</v>
       </c>
       <c r="C5" s="10" t="n">
-        <v>1300</v>
+        <v>1100</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>48</v>
@@ -1449,7 +1449,7 @@
       <c r="B10" s="15"/>
       <c r="C10" s="16" t="n">
         <f aca="false">SUM(C5:C9)</f>
-        <v>1500</v>
+        <v>1300</v>
       </c>
       <c r="D10" s="15"/>
     </row>
@@ -1525,14 +1525,14 @@
       </c>
       <c r="D5" s="17" t="n">
         <f aca="false">ROUND(C5*(1+Premissas!$B$6),0)</f>
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E5" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F5" s="9" t="n">
         <f aca="false">(D5*Premissas!$B$5+E5)*(1+Premissas!$B$12)</f>
-        <v>21440</v>
+        <v>21120</v>
       </c>
       <c r="G5" s="4"/>
     </row>
@@ -1544,18 +1544,18 @@
         <v>68</v>
       </c>
       <c r="C6" s="12" t="n">
-        <v>240</v>
+        <v>200</v>
       </c>
       <c r="D6" s="17" t="n">
         <f aca="false">ROUND(C6*(1+Premissas!$B$6),0)</f>
-        <v>269</v>
+        <v>220</v>
       </c>
       <c r="E6" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F6" s="9" t="n">
         <f aca="false">(D6*Premissas!$B$5+E6)*(1+Premissas!$B$12)</f>
-        <v>43040</v>
+        <v>35200</v>
       </c>
       <c r="G6" s="4"/>
     </row>
@@ -1567,18 +1567,18 @@
         <v>69</v>
       </c>
       <c r="C7" s="12" t="n">
-        <v>200</v>
+        <v>180</v>
       </c>
       <c r="D7" s="17" t="n">
         <f aca="false">ROUND(C7*(1+Premissas!$B$6),0)</f>
-        <v>224</v>
+        <v>198</v>
       </c>
       <c r="E7" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F7" s="9" t="n">
         <f aca="false">(D7*Premissas!$B$5+E7)*(1+Premissas!$B$12)</f>
-        <v>35840</v>
+        <v>31680</v>
       </c>
       <c r="G7" s="4" t="s">
         <v>70</v>
@@ -1592,18 +1592,18 @@
         <v>71</v>
       </c>
       <c r="C8" s="12" t="n">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="D8" s="17" t="n">
         <f aca="false">ROUND(C8*(1+Premissas!$B$6),0)</f>
-        <v>246</v>
+        <v>231</v>
       </c>
       <c r="E8" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F8" s="9" t="n">
         <f aca="false">(D8*Premissas!$B$5+E8)*(1+Premissas!$B$12)</f>
-        <v>39360</v>
+        <v>36960</v>
       </c>
       <c r="G8" s="4" t="s">
         <v>72</v>
@@ -1617,18 +1617,18 @@
         <v>73</v>
       </c>
       <c r="C9" s="12" t="n">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="D9" s="17" t="n">
         <f aca="false">ROUND(C9*(1+Premissas!$B$6),0)</f>
-        <v>246</v>
+        <v>231</v>
       </c>
       <c r="E9" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="9" t="n">
         <f aca="false">(D9*Premissas!$B$5+E9)*(1+Premissas!$B$12)</f>
-        <v>39360</v>
+        <v>36960</v>
       </c>
       <c r="G9" s="4" t="s">
         <v>74</v>
@@ -1646,14 +1646,14 @@
       </c>
       <c r="D10" s="17" t="n">
         <f aca="false">ROUND(C10*(1+Premissas!$B$6),0)</f>
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E10" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="9" t="n">
         <f aca="false">(D10*Premissas!$B$5+E10)*(1+Premissas!$B$12)</f>
-        <v>14400</v>
+        <v>14080</v>
       </c>
       <c r="G10" s="4"/>
     </row>
@@ -1665,18 +1665,18 @@
         <v>76</v>
       </c>
       <c r="C11" s="12" t="n">
-        <v>200</v>
+        <v>180</v>
       </c>
       <c r="D11" s="17" t="n">
         <f aca="false">ROUND(C11*(1+Premissas!$B$6),0)</f>
-        <v>224</v>
+        <v>198</v>
       </c>
       <c r="E11" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F11" s="9" t="n">
         <f aca="false">(D11*Premissas!$B$5+E11)*(1+Premissas!$B$12)</f>
-        <v>35840</v>
+        <v>31680</v>
       </c>
       <c r="G11" s="4" t="s">
         <v>77</v>
@@ -1694,14 +1694,14 @@
       </c>
       <c r="D12" s="17" t="n">
         <f aca="false">ROUND(C12*(1+Premissas!$B$6),0)</f>
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E12" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="9" t="n">
         <f aca="false">(D12*Premissas!$B$5+E12)*(1+Premissas!$B$12)</f>
-        <v>10720</v>
+        <v>10560</v>
       </c>
       <c r="G12" s="4"/>
     </row>
@@ -1717,14 +1717,14 @@
       </c>
       <c r="D13" s="17" t="n">
         <f aca="false">ROUND(C13*(1+Premissas!$B$6),0)</f>
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E13" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="9" t="n">
         <f aca="false">(D13*Premissas!$B$5+E13)*(1+Premissas!$B$12)</f>
-        <v>17920</v>
+        <v>17600</v>
       </c>
       <c r="G13" s="4"/>
     </row>
@@ -1736,18 +1736,18 @@
         <v>80</v>
       </c>
       <c r="C14" s="12" t="n">
-        <v>200</v>
+        <v>180</v>
       </c>
       <c r="D14" s="17" t="n">
         <f aca="false">ROUND(C14*(1+Premissas!$B$6),0)</f>
-        <v>224</v>
+        <v>198</v>
       </c>
       <c r="E14" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F14" s="9" t="n">
         <f aca="false">(D14*Premissas!$B$5+E14)*(1+Premissas!$B$12)</f>
-        <v>35840</v>
+        <v>31680</v>
       </c>
       <c r="G14" s="4"/>
     </row>
@@ -1759,18 +1759,18 @@
         <v>81</v>
       </c>
       <c r="C15" s="12" t="n">
-        <v>160</v>
+        <v>140</v>
       </c>
       <c r="D15" s="17" t="n">
         <f aca="false">ROUND(C15*(1+Premissas!$B$6),0)</f>
-        <v>179</v>
+        <v>154</v>
       </c>
       <c r="E15" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F15" s="9" t="n">
         <f aca="false">(D15*Premissas!$B$5+E15)*(1+Premissas!$B$12)</f>
-        <v>28640</v>
+        <v>24640</v>
       </c>
       <c r="G15" s="4" t="s">
         <v>82</v>
@@ -1784,18 +1784,18 @@
         <v>83</v>
       </c>
       <c r="C16" s="12" t="n">
-        <v>240</v>
+        <v>200</v>
       </c>
       <c r="D16" s="17" t="n">
         <f aca="false">ROUND(C16*(1+Premissas!$B$6),0)</f>
-        <v>269</v>
+        <v>220</v>
       </c>
       <c r="E16" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F16" s="9" t="n">
         <f aca="false">(D16*Premissas!$B$5+E16)*(1+Premissas!$B$12)</f>
-        <v>43040</v>
+        <v>35200</v>
       </c>
       <c r="G16" s="4"/>
     </row>
@@ -1811,14 +1811,14 @@
       </c>
       <c r="D17" s="17" t="n">
         <f aca="false">ROUND(C17*(1+Premissas!$B$6),0)</f>
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="E17" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F17" s="9" t="n">
         <f aca="false">(D17*Premissas!$B$5+E17)*(1+Premissas!$B$12)</f>
-        <v>25120</v>
+        <v>24640</v>
       </c>
       <c r="G17" s="4"/>
     </row>
@@ -1834,14 +1834,14 @@
       </c>
       <c r="D18" s="17" t="n">
         <f aca="false">ROUND(C18*(1+Premissas!$B$6),0)</f>
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E18" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F18" s="9" t="n">
         <f aca="false">(D18*Premissas!$B$5+E18)*(1+Premissas!$B$12)</f>
-        <v>17920</v>
+        <v>17600</v>
       </c>
       <c r="G18" s="4"/>
     </row>
@@ -1853,18 +1853,18 @@
         <v>86</v>
       </c>
       <c r="C19" s="12" t="n">
-        <v>200</v>
+        <v>180</v>
       </c>
       <c r="D19" s="17" t="n">
         <f aca="false">ROUND(C19*(1+Premissas!$B$6),0)</f>
-        <v>224</v>
+        <v>198</v>
       </c>
       <c r="E19" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F19" s="9" t="n">
         <f aca="false">(D19*Premissas!$B$5+E19)*(1+Premissas!$B$12)</f>
-        <v>35840</v>
+        <v>31680</v>
       </c>
       <c r="G19" s="4"/>
     </row>
@@ -1876,18 +1876,18 @@
         <v>87</v>
       </c>
       <c r="C20" s="12" t="n">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="D20" s="17" t="n">
         <f aca="false">ROUND(C20*(1+Premissas!$B$6),0)</f>
-        <v>134</v>
+        <v>121</v>
       </c>
       <c r="E20" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F20" s="9" t="n">
         <f aca="false">(D20*Premissas!$B$5+E20)*(1+Premissas!$B$12)</f>
-        <v>21440</v>
+        <v>19360</v>
       </c>
       <c r="G20" s="4"/>
     </row>
@@ -1903,7 +1903,7 @@
       </c>
       <c r="D21" s="17" t="n">
         <f aca="false">ROUND(C21*(1+Premissas!$B$6),0)</f>
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E21" s="5" t="n">
         <f aca="false">Premissas!$B$7</f>
@@ -1911,7 +1911,7 @@
       </c>
       <c r="F21" s="9" t="n">
         <f aca="false">(D21*Premissas!$B$5+E21)*(1+Premissas!$B$12)</f>
-        <v>16720</v>
+        <v>16560</v>
       </c>
       <c r="G21" s="4" t="s">
         <v>89</v>
@@ -1924,11 +1924,11 @@
       </c>
       <c r="C22" s="19" t="n">
         <f aca="false">SUM(C5:C21)</f>
-        <v>2660</v>
+        <v>2450</v>
       </c>
       <c r="D22" s="19" t="n">
         <f aca="false">SUM(D5:D21)</f>
-        <v>2978</v>
+        <v>2695</v>
       </c>
       <c r="E22" s="16" t="n">
         <f aca="false">SUM(E5:E21)</f>
@@ -1936,7 +1936,7 @@
       </c>
       <c r="F22" s="16" t="n">
         <f aca="false">SUM(F5:F21)</f>
-        <v>482480</v>
+        <v>437200</v>
       </c>
       <c r="G22" s="15"/>
     </row>
@@ -1972,7 +1972,7 @@
       </c>
       <c r="C25" s="5" t="n">
         <f aca="false">Nuvem!$C$10</f>
-        <v>1500</v>
+        <v>1300</v>
       </c>
       <c r="D25" s="8" t="n">
         <f aca="false">Premissas!$B$8</f>
@@ -1980,11 +1980,11 @@
       </c>
       <c r="E25" s="9" t="n">
         <f aca="false">(C25)*(1+Premissas!$B$12)</f>
-        <v>1500</v>
+        <v>1300</v>
       </c>
       <c r="F25" s="9" t="n">
         <f aca="false">E25*D25</f>
-        <v>36000</v>
+        <v>31200</v>
       </c>
       <c r="G25" s="4" t="s">
         <v>97</v>
@@ -1999,7 +1999,7 @@
       </c>
       <c r="C26" s="8" t="n">
         <f aca="false">Premissas!$B$9</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D26" s="8" t="n">
         <f aca="false">Premissas!$B$8</f>
@@ -2007,11 +2007,11 @@
       </c>
       <c r="E26" s="9" t="n">
         <f aca="false">(C26*Premissas!$B$5+Premissas!$B$10)*(1+Premissas!$B$12)</f>
-        <v>800</v>
+        <v>640</v>
       </c>
       <c r="F26" s="9" t="n">
         <f aca="false">E26*D26</f>
-        <v>19200</v>
+        <v>15360</v>
       </c>
       <c r="G26" s="4" t="s">
         <v>99</v>
@@ -2026,7 +2026,7 @@
       </c>
       <c r="C27" s="8" t="n">
         <f aca="false">Premissas!$B$11</f>
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="D27" s="8" t="n">
         <f aca="false">Premissas!$B$8</f>
@@ -2034,11 +2034,11 @@
       </c>
       <c r="E27" s="9" t="n">
         <f aca="false">(C27*Premissas!$B$5)*(1+Premissas!$B$12)</f>
-        <v>3200</v>
+        <v>2400</v>
       </c>
       <c r="F27" s="9" t="n">
         <f aca="false">E27*D27</f>
-        <v>76800</v>
+        <v>57600</v>
       </c>
       <c r="G27" s="4" t="s">
         <v>101</v>
@@ -2053,11 +2053,11 @@
       <c r="D28" s="15"/>
       <c r="E28" s="16" t="n">
         <f aca="false">SUM(E25:E27)</f>
-        <v>5500</v>
+        <v>4340</v>
       </c>
       <c r="F28" s="16" t="n">
         <f aca="false">SUM(F25:F27)</f>
-        <v>132000</v>
+        <v>104160</v>
       </c>
       <c r="G28" s="15"/>
     </row>
@@ -2067,7 +2067,7 @@
       </c>
       <c r="F30" s="7" t="n">
         <f aca="false">F22+F28</f>
-        <v>614480</v>
+        <v>541360</v>
       </c>
     </row>
   </sheetData>
@@ -2123,15 +2123,15 @@
         <v>109</v>
       </c>
       <c r="B5" s="12" t="n">
-        <v>320</v>
+        <v>245</v>
       </c>
       <c r="C5" s="20" t="n">
         <f aca="false">IFERROR(B5/$B$11,0)</f>
-        <v>0.107454667562122</v>
+        <v>0.0909090909090909</v>
       </c>
       <c r="D5" s="9" t="n">
         <f aca="false">B5*Premissas!$B$5</f>
-        <v>51200</v>
+        <v>39200</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2139,15 +2139,15 @@
         <v>110</v>
       </c>
       <c r="B6" s="12" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="C6" s="20" t="n">
         <f aca="false">IFERROR(B6/$B$11,0)</f>
-        <v>0.151108126259234</v>
+        <v>0.155844155844156</v>
       </c>
       <c r="D6" s="9" t="n">
         <f aca="false">B6*Premissas!$B$5</f>
-        <v>72000</v>
+        <v>67200</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2155,15 +2155,15 @@
         <v>111</v>
       </c>
       <c r="B7" s="12" t="n">
-        <v>1400</v>
+        <v>1270</v>
       </c>
       <c r="C7" s="20" t="n">
         <f aca="false">IFERROR(B7/$B$11,0)</f>
-        <v>0.470114170584285</v>
+        <v>0.471243042671614</v>
       </c>
       <c r="D7" s="9" t="n">
         <f aca="false">B7*Premissas!$B$5</f>
-        <v>224000</v>
+        <v>203200</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2171,15 +2171,15 @@
         <v>112</v>
       </c>
       <c r="B8" s="12" t="n">
-        <v>350</v>
+        <v>300</v>
       </c>
       <c r="C8" s="20" t="n">
         <f aca="false">IFERROR(B8/$B$11,0)</f>
-        <v>0.117528542646071</v>
+        <v>0.111317254174397</v>
       </c>
       <c r="D8" s="9" t="n">
         <f aca="false">B8*Premissas!$B$5</f>
-        <v>56000</v>
+        <v>48000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2187,15 +2187,15 @@
         <v>113</v>
       </c>
       <c r="B9" s="12" t="n">
-        <v>300</v>
+        <v>290</v>
       </c>
       <c r="C9" s="20" t="n">
         <f aca="false">IFERROR(B9/$B$11,0)</f>
-        <v>0.10073875083949</v>
+        <v>0.10760667903525</v>
       </c>
       <c r="D9" s="9" t="n">
         <f aca="false">B9*Premissas!$B$5</f>
-        <v>48000</v>
+        <v>46400</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2203,15 +2203,15 @@
         <v>114</v>
       </c>
       <c r="B10" s="12" t="n">
-        <v>158</v>
+        <v>170</v>
       </c>
       <c r="C10" s="20" t="n">
         <f aca="false">IFERROR(B10/$B$11,0)</f>
-        <v>0.0530557421087979</v>
+        <v>0.0630797773654917</v>
       </c>
       <c r="D10" s="9" t="n">
         <f aca="false">B10*Premissas!$B$5</f>
-        <v>25280</v>
+        <v>27200</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2220,7 +2220,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="false">SUM(B5:B10)</f>
-        <v>2978</v>
+        <v>2695</v>
       </c>
       <c r="C11" s="21" t="n">
         <f aca="false">SUM(C5:C10)</f>
@@ -2228,7 +2228,7 @@
       </c>
       <c r="D11" s="16" t="n">
         <f aca="false">SUM(D5:D10)</f>
-        <v>476480</v>
+        <v>431200</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2237,7 +2237,7 @@
       </c>
       <c r="B12" s="8" t="n">
         <f aca="false">Componentes!$D$22</f>
-        <v>2978</v>
+        <v>2695</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2309,7 +2309,7 @@
       </c>
       <c r="D5" s="9" t="n">
         <f aca="false">C5*Componentes!$F$22</f>
-        <v>48248</v>
+        <v>43720</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2324,7 +2324,7 @@
       </c>
       <c r="D6" s="9" t="n">
         <f aca="false">C6*Componentes!$F$22</f>
-        <v>72372</v>
+        <v>65580</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2339,7 +2339,7 @@
       </c>
       <c r="D7" s="9" t="n">
         <f aca="false">C7*Componentes!$F$22</f>
-        <v>96496</v>
+        <v>87440</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2354,7 +2354,7 @@
       </c>
       <c r="D8" s="9" t="n">
         <f aca="false">C8*Componentes!$F$22</f>
-        <v>96496</v>
+        <v>87440</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2369,7 +2369,7 @@
       </c>
       <c r="D9" s="9" t="n">
         <f aca="false">C9*Componentes!$F$22</f>
-        <v>96496</v>
+        <v>87440</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2384,7 +2384,7 @@
       </c>
       <c r="D10" s="9" t="n">
         <f aca="false">C10*Componentes!$F$22</f>
-        <v>72372</v>
+        <v>65580</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2398,7 +2398,7 @@
       </c>
       <c r="D11" s="16" t="n">
         <f aca="false">SUM(D5:D10)</f>
-        <v>482480</v>
+        <v>437200</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2407,7 +2407,7 @@
       </c>
       <c r="D13" s="5" t="n">
         <f aca="false">Componentes!$E$28</f>
-        <v>5500</v>
+        <v>4340</v>
       </c>
     </row>
   </sheetData>

</xml_diff>